<commit_message>
Import 4 vials from CAA Lab-Cell Stocks (-80 & LiqNitro)-2 NEW.xlsx from umut-PC
</commit_message>
<xml_diff>
--- a/cellstocks/data/caa.xlsx
+++ b/cellstocks/data/caa.xlsx
@@ -161,7 +161,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box 1</t>
+          <t xml:space="preserve">CLAUDE BOX 1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -238,7 +238,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box 1</t>
+          <t xml:space="preserve">CLAUDE BOX 1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -299,6 +299,160 @@
       <c r="S3" t="inlineStr">
         <is>
           <t xml:space="preserve">v-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-80 °C Freezer</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fff</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCAP</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-28</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28-07-25</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-83</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-80 °C Freezer</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fff</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lncap caspex</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-28</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28-07-25</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-84</t>
         </is>
       </c>
     </row>
@@ -349,22 +503,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek caspex g8</t>
+          <t xml:space="preserve">LNCAP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">g8</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E2">
@@ -380,7 +534,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">hek tox4 KO g8</t>
+          <t xml:space="preserve">hek caspex g8</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -390,7 +544,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -405,6 +559,68 @@
         <v>0</v>
       </c>
       <c r="G3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hek tox4 KO g8</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KO</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g8</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lncap caspex</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
         <v>1</v>
       </c>
     </row>
@@ -544,7 +760,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box 1</t>
+          <t xml:space="preserve">CLAUDE BOX 1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -565,6 +781,48 @@
         <v>2</v>
       </c>
       <c r="J2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-80 °C Freezer</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">freezer</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fff</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F3">
+        <v>9</v>
+      </c>
+      <c r="G3">
+        <v>9</v>
+      </c>
+      <c r="H3">
+        <v>81</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
         <v>79</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Edit LNCAP from Umut iphone cell stocks
</commit_message>
<xml_diff>
--- a/cellstocks/data/caa.xlsx
+++ b/cellstocks/data/caa.xlsx
@@ -328,9 +328,14 @@
           <t xml:space="preserve">LNCAP</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p5</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">

</xml_diff>

<commit_message>
Edit hek caspex g8 from Umut iphone cell stocks
</commit_message>
<xml_diff>
--- a/cellstocks/data/caa.xlsx
+++ b/cellstocks/data/caa.xlsx
@@ -174,9 +174,14 @@
           <t xml:space="preserve">hek caspex g8</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P6</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
Edit hek tox4 KO g8 from Umut iphone cell stocks
</commit_message>
<xml_diff>
--- a/cellstocks/data/caa.xlsx
+++ b/cellstocks/data/caa.xlsx
@@ -256,9 +256,14 @@
           <t xml:space="preserve">hek tox4 KO g8</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P5</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">

</xml_diff>

<commit_message>
Edit lncap caspex from Umut iphone cell stocks
</commit_message>
<xml_diff>
--- a/cellstocks/data/caa.xlsx
+++ b/cellstocks/data/caa.xlsx
@@ -420,9 +420,14 @@
           <t xml:space="preserve">lncap caspex</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P6</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">

</xml_diff>